<commit_message>
Remove bounced emails from roller hockey clubs list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TQQnwrTZ1Rgq1vjwXmKstT
</commit_message>
<xml_diff>
--- a/hoquei/clubs_hoquei_patins_catalunya.xlsx
+++ b/hoquei/clubs_hoquei_patins_catalunya.xlsx
@@ -481,28 +481,28 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Cambrils Club Hoquei</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Cambrils</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>cambrilsclubhoquei@gmail.com</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>cambrilsch.cat</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Correu rebotat eliminat: cambrilsclubhoquei@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -933,26 +933,22 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Club Hoquei Esplugues</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Esplugues de Llobregat</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>seniorhce@gmail.com</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>tel 93 473 1899</t>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>tel 93 473 1899 · Correu rebotat eliminat: seniorhce@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1149,34 +1145,30 @@
       <c r="F25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Club Hoquei Palafrugell</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Palafrugell</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>info@chpalafrugell.cat</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>chpalafrugell.cat</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>@chpalafrugell (X)</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>tel 972612449</t>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>tel 972612449 · Correu rebotat eliminat: info@chpalafrugell.cat</t>
         </is>
       </c>
     </row>
@@ -1745,26 +1737,22 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>Club Patí Riudoms</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Riudoms</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>info@clubpatiriudoms.com; info@cpriudoms.club</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr"/>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>tel 628101216</t>
+      <c r="C47" s="3" t="n"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>tel 628101216 · Correu rebotat eliminat: info@clubpatiriudoms.com, info@cpriudoms.club</t>
         </is>
       </c>
     </row>
@@ -1969,30 +1957,26 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Club Patí Vilafranca</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Vilafranca del Penedès</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>hello@cpvilafranca.cat</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="C55" s="3" t="n"/>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>cpvilafranca.cat</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr"/>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>tel 93 817 31 31</t>
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>tel 93 817 31 31 · Correu rebotat eliminat: hello@cpvilafranca.cat</t>
         </is>
       </c>
     </row>
@@ -2025,26 +2009,22 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Club Sants-Montjuïc Hoquei Patins</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Barcelona</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>santsmontjuic@esportbarrio.com</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr"/>
-      <c r="E57" s="2" t="inlineStr"/>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>tel 934910549</t>
+      <c r="C57" s="3" t="n"/>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>tel 934910549 · Correu rebotat eliminat: santsmontjuic@esportbarrio.com</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2069,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>info@reusploms.cat; actividades@reusploms.cat</t>
+          <t>info@reusploms.cat</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2098,7 +2078,11 @@
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Correu rebotat eliminat: actividades@reusploms.cat</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2729,34 +2713,30 @@
       <c r="F81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>Patí Hoquei Club Sant Cugat</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>Sant Cugat del Vallès</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>santcugat-ok.campus@hotmail.com</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="C82" s="3" t="n"/>
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>phcsantcugat.com</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
+      <c r="E82" s="3" t="inlineStr">
         <is>
           <t>@phcsantcugat (X)</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>tel 699 076 123</t>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>tel 699 076 123 · Correu rebotat eliminat: santcugat-ok.campus@hotmail.com</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3344,41 +3324,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>cambrilsclubhoquei@gmail.com</t>
+          <t>kphoqueiclub@gmail.com</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cambrils Club Hoquei</t>
+          <t>Capellades Hoquei Club</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cambrils</t>
+          <t>Capellades</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>kphoqueiclub@gmail.com</t>
+          <t>cecornellacoordinacio@gmail.com</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Capellades Hoquei Club</t>
+          <t>CE Cornellà (hoquei patins)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Capellades</t>
+          <t>Cornellà de Llobregat</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cecornellacoordinacio@gmail.com</t>
+          <t>cornellahockeypatines@gmail.com</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3395,41 +3375,41 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cornellahockeypatines@gmail.com</t>
+          <t>club@lleida-llista.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CE Cornellà (hoquei patins)</t>
+          <t>CE Lleida Llista Blava</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cornellà de Llobregat</t>
+          <t>Lleida</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>club@lleida-llista.com</t>
+          <t>hoquei@cenoia.com</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CE Lleida Llista Blava</t>
+          <t>CE Noia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Lleida</t>
+          <t>Sant Sadurní d'Anoia</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>hoquei@cenoia.com</t>
+          <t>comunicacio@cenoia.com</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3446,7 +3426,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>comunicacio@cenoia.com</t>
+          <t>cenoia@cenoia.com</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3463,24 +3443,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cenoia@cenoia.com</t>
+          <t>info@olimpicreus.cat</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CE Noia</t>
+          <t>CEH Olímpic Reus</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sant Sadurní d'Anoia</t>
+          <t>Reus</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>info@olimpicreus.cat</t>
+          <t>hoqueiolimpicreus@gmail.com</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3497,24 +3477,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>hoqueiolimpicreus@gmail.com</t>
+          <t>info@cerdanyolach.com</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CEH Olímpic Reus</t>
+          <t>Cerdanyola Club Hoquei</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Reus</t>
+          <t>Cerdanyola del Vallès</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>info@cerdanyolach.com</t>
+          <t>cerdanyolaclubhoquei@fecapa.cat</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3531,24 +3511,24 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cerdanyolaclubhoquei@fecapa.cat</t>
+          <t>info@chcaldes.com</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cerdanyola Club Hoquei</t>
+          <t>CH Caldes</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cerdanyola del Vallès</t>
+          <t>Caldes de Montbui</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>info@chcaldes.com</t>
+          <t>chcaldes@gmail.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3565,7 +3545,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>chcaldes@gmail.com</t>
+          <t>premsachcaldes@gmail.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3582,143 +3562,143 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>premsachcaldes@gmail.com</t>
+          <t>secretaria@hoqueibiguesiriells.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CH Caldes</t>
+          <t>CHP Bigues i Riells</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Caldes de Montbui</t>
+          <t>Bigues i Riells</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>secretaria@hoqueibiguesiriells.com</t>
+          <t>info@chpsantfeliu.cat</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CHP Bigues i Riells</t>
+          <t>CHP Sant Feliu de Codines</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Bigues i Riells</t>
+          <t>Sant Feliu de Codines</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>info@chpsantfeliu.cat</t>
+          <t>comunicacio@hoqueicadi.cat</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CHP Sant Feliu de Codines</t>
+          <t>CHPA Cadí</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sant Feliu de Codines</t>
+          <t>La Seu d'Urgell</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>comunicacio@hoqueicadi.cat</t>
+          <t>joanestevecasablancas@gmail.com</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CHPA Cadí</t>
+          <t>Club Esportiu Hoquei Sabadell</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>La Seu d'Urgell</t>
+          <t>Sabadell</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>joanestevecasablancas@gmail.com</t>
+          <t>hoqueiarenysdemar@gmail.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Club Esportiu Hoquei Sabadell</t>
+          <t>Club Hoquei Arenys de Mar</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sabadell</t>
+          <t>Arenys de Mar</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>hoqueiarenysdemar@gmail.com</t>
+          <t>info@casaldelespluga.cat</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Club Hoquei Arenys de Mar</t>
+          <t>Club Hoquei Casal Espluga</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Arenys de Mar</t>
+          <t>L'Espluga de Francolí</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>info@casaldelespluga.cat</t>
+          <t>castellethoquei@gmail.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Club Hoquei Casal Espluga</t>
+          <t>Club Hoquei Castellet</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>L'Espluga de Francolí</t>
+          <t>Sant Vicenç de Castellet</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>castellethoquei@gmail.com</t>
+          <t>info@hoqueiclaret.com</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Club Hoquei Castellet</t>
+          <t>Club Hoquei Claret Barcelona</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sant Vicenç de Castellet</t>
+          <t>Barcelona</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>info@hoqueiclaret.com</t>
+          <t>inscripcions@hoqueiclaret.com</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3735,1409 +3715,1256 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>inscripcions@hoqueiclaret.com</t>
+          <t>hoqueifigueres@yahoo.es</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Club Hoquei Claret Barcelona</t>
+          <t>Club Hoquei Figueres</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Figueres</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>seniorhce@gmail.com</t>
+          <t>info@hoqueilesfranqueses.cat</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Club Hoquei Esplugues</t>
+          <t>Club Hoquei Les Franqueses</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Esplugues de Llobregat</t>
+          <t>Les Franqueses del Vallès</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>hoqueifigueres@yahoo.es</t>
+          <t>info@hoqueilloret.org</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Club Hoquei Figueres</t>
+          <t>Club Hoquei Lloret</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Figueres</t>
+          <t>Lloret de Mar</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>info@hoqueilesfranqueses.cat</t>
+          <t>okmolins@gmail.com</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Club Hoquei Les Franqueses</t>
+          <t>Club Hoquei Molins de Rei</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Les Franqueses del Vallès</t>
+          <t>Molins de Rei</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>info@hoqueilloret.org</t>
+          <t>chmollerussa@gmail.com</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Club Hoquei Lloret</t>
+          <t>Club Hoquei Mollerussa</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Lloret de Mar</t>
+          <t>Mollerussa</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>okmolins@gmail.com</t>
+          <t>clubhoqueinavarcles@gmail.com</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Club Hoquei Molins de Rei</t>
+          <t>Club Hoquei Navarcles</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Molins de Rei</t>
+          <t>Navarcles</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>chmollerussa@gmail.com</t>
+          <t>hoqueiolot@gmail.com</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Club Hoquei Mollerussa</t>
+          <t>Club Hoquei Olot</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mollerussa</t>
+          <t>Olot</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>clubhoqueinavarcles@gmail.com</t>
+          <t>hoqueipatinsmartorell@gmail.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Club Hoquei Navarcles</t>
+          <t>Club Hoquei Patins Martorell</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Navarcles</t>
+          <t>Martorell</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>hoqueiolot@gmail.com</t>
+          <t>comunicacio@hoqueibadalona.cat</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Club Hoquei Olot</t>
+          <t>Club Hoquei Patí Sant Josep de Badalona</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Olot</t>
+          <t>Badalona</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>info@chpalafrugell.cat</t>
+          <t>lopd@hoqueibadalona.cat</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Club Hoquei Palafrugell</t>
+          <t>Club Hoquei Patí Sant Josep de Badalona</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Palafrugell</t>
+          <t>Badalona</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>hoqueipatinsmartorell@gmail.com</t>
+          <t>chpremia@gmail.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Club Hoquei Patins Martorell</t>
+          <t>Club Hoquei Premià</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Martorell</t>
+          <t>Premià de Mar</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>comunicacio@hoqueibadalona.cat</t>
+          <t>info@clubhoqueiripollet.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Club Hoquei Patí Sant Josep de Badalona</t>
+          <t>Club Hoquei Ripollet</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Badalona</t>
+          <t>Ripollet</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>lopd@hoqueibadalona.cat</t>
+          <t>hoqueisantjordi@gmail.com</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Club Hoquei Patí Sant Josep de Badalona</t>
+          <t>Club Hoquei Sant Jordi Desvalls</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Badalona</t>
+          <t>Sant Jordi Desvalls</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>chpremia@gmail.com</t>
+          <t>clubhoqueisantaperpetua@gmail.com</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Club Hoquei Premià</t>
+          <t>Club Hoquei Santa Perpètua</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Premià de Mar</t>
+          <t>Santa Perpètua de Mogoda</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>info@clubhoqueiripollet.com</t>
+          <t>clubhoqueisantaperpetua@fecapa.cat</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Club Hoquei Ripollet</t>
+          <t>Club Hoquei Santa Perpètua</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Ripollet</t>
+          <t>Santa Perpètua de Mogoda</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>hoqueisantjordi@gmail.com</t>
+          <t>info@chvs.cat</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Club Hoquei Sant Jordi Desvalls</t>
+          <t>Club Hoquei Vila-seca</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Sant Jordi Desvalls</t>
+          <t>Vila-seca</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>clubhoqueisantaperpetua@gmail.com</t>
+          <t>clubhoqueivilaseca@fecapa.cat</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Club Hoquei Santa Perpètua</t>
+          <t>Club Hoquei Vila-seca</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Santa Perpètua de Mogoda</t>
+          <t>Vila-seca</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>clubhoqueisantaperpetua@fecapa.cat</t>
+          <t>clubpatialcover@gmail.com</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Club Hoquei Santa Perpètua</t>
+          <t>Club Patí Alcover</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Santa Perpètua de Mogoda</t>
+          <t>Alcover</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>info@chvs.cat</t>
+          <t>cpbell.lloc@gmail.com</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Club Hoquei Vila-seca</t>
+          <t>Club Patí Bell-lloc</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Vila-seca</t>
+          <t>Bell-lloc d'Urgell</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>clubhoqueivilaseca@fecapa.cat</t>
+          <t>cpblanes2015@gmail.com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Club Hoquei Vila-seca</t>
+          <t>Club Patí Blanes Atlètic</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Vila-seca</t>
+          <t>Blanes</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>clubpatialcover@gmail.com</t>
+          <t>clubpaticabrils@gmail.com</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Club Patí Alcover</t>
+          <t>Club Patí Cabrils</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Alcover</t>
+          <t>Cabrils</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cpbell.lloc@gmail.com</t>
+          <t>cpcalafell@cpcalafell.com</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Club Patí Bell-lloc</t>
+          <t>Club Patí Calafell</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Bell-lloc d'Urgell</t>
+          <t>Calafell</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>cpblanes2015@gmail.com</t>
+          <t>clubpaticentelles@fecapa.cat</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Club Patí Blanes Atlètic</t>
+          <t>Club Patí Centelles</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Blanes</t>
+          <t>Centelles</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>clubpaticabrils@gmail.com</t>
+          <t>info_hoquei@cpcongres.cat</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Club Patí Cabrils</t>
+          <t>Club Patí Congrés</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Cabrils</t>
+          <t>Barcelona</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>cpcalafell@cpcalafell.com</t>
+          <t>hoqueibasecpcongres@gmail.com</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Club Patí Calafell</t>
+          <t>Club Patí Congrés</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Calafell</t>
+          <t>Barcelona</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>clubpaticentelles@fecapa.cat</t>
+          <t>clubpaticorbera@fecapa.cat</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Club Patí Centelles</t>
+          <t>Club Patí Corbera</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Centelles</t>
+          <t>Corbera de Llobregat</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>info_hoquei@cpcongres.cat</t>
+          <t>clubpatifolgueroles@fecapa.cat</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Club Patí Congrés</t>
+          <t>Club Patí Folgueroles</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Folgueroles</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>hoqueibasecpcongres@gmail.com</t>
+          <t>cpgramenet@gmail.com</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Club Patí Congrés</t>
+          <t>Club Patí Gramenet</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Santa Coloma de Gramenet</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>clubpaticorbera@fecapa.cat</t>
+          <t>clubpatimalgrat@gmail.com</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Club Patí Corbera</t>
+          <t>Club Patí Malgrat</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Corbera de Llobregat</t>
+          <t>Malgrat de Mar</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>clubpatifolgueroles@fecapa.cat</t>
+          <t>clubpatimanresahoquei@gmail.com</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Club Patí Folgueroles</t>
+          <t>Club Patí Manresa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Folgueroles</t>
+          <t>Manresa</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>cpgramenet@gmail.com</t>
+          <t>secretaria@clubpatimanresa.cat</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Club Patí Gramenet</t>
+          <t>Club Patí Manresa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Santa Coloma de Gramenet</t>
+          <t>Manresa</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>clubpatimalgrat@gmail.com</t>
+          <t>clubpatinatgeparets@gmail.com</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Club Patí Malgrat</t>
+          <t>Club Patí Parets</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Malgrat de Mar</t>
+          <t>Parets del Vallès</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>clubpatimanresahoquei@gmail.com</t>
+          <t>cprodahoquei@gmail.com</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Club Patí Manresa</t>
+          <t>Club Patí Roda</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Manresa</t>
+          <t>Roda de Ter</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>secretaria@clubpatimanresa.cat</t>
+          <t>angels.ventura@gmail.com</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Club Patí Manresa</t>
+          <t>Club Patí Sant Ramon</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Manresa</t>
+          <t>Vilafranca del Penedès</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>clubpatinatgeparets@gmail.com</t>
+          <t>hoquei@clubpatisitges.com</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Club Patí Parets</t>
+          <t>Club Patí Sitges</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Parets del Vallès</t>
+          <t>Sitges</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>info@clubpatiriudoms.com</t>
+          <t>admin@cptaradell.cat</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Club Patí Riudoms</t>
+          <t>Club Patí Taradell</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Riudoms</t>
+          <t>Taradell</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>info@cpriudoms.club</t>
+          <t>cptordera0910@gmail.com</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Club Patí Riudoms</t>
+          <t>Club Patí Tordera</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Riudoms</t>
+          <t>Tordera</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>cprodahoquei@gmail.com</t>
+          <t>clubpatitorrelles@gmail.com</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Club Patí Roda</t>
+          <t>Club Patí Torrelles</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Roda de Ter</t>
+          <t>Torrelles de Llobregat</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>angels.ventura@gmail.com</t>
+          <t>info@clubpativic.cat</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Club Patí Sant Ramon</t>
+          <t>Club Patí Vic</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Vilafranca del Penedès</t>
+          <t>Vic</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>hoquei@clubpatisitges.com</t>
+          <t>cpvilanova@clubpativilanovafundacio.cat</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Club Patí Sitges</t>
+          <t>Club Patí Vilanova</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sitges</t>
+          <t>Vilanova i la Geltrú</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>admin@cptaradell.cat</t>
+          <t>admin@vilassarhoquei.cat</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Club Patí Taradell</t>
+          <t>Club Vilassar Hoquei</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Taradell</t>
+          <t>Vilassar de Mar</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>cptordera0910@gmail.com</t>
+          <t>esportiu@vilassarhoquei.cat</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Club Patí Tordera</t>
+          <t>Club Vilassar Hoquei</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Tordera</t>
+          <t>Vilassar de Mar</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>clubpatitorrelles@gmail.com</t>
+          <t>web@vilassarhoquei.cat</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Club Patí Torrelles</t>
+          <t>Club Vilassar Hoquei</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Torrelles de Llobregat</t>
+          <t>Vilassar de Mar</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>info@clubpativic.cat</t>
+          <t>sponsors@vilassarhoquei.cat</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Club Patí Vic</t>
+          <t>Club Vilassar Hoquei</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Vic</t>
+          <t>Vilassar de Mar</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>hello@cpvilafranca.cat</t>
+          <t>equipacions@vilassarhoquei.cat</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Club Patí Vilafranca</t>
+          <t>Club Vilassar Hoquei</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Vilafranca del Penedès</t>
+          <t>Vilassar de Mar</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>cpvilanova@clubpativilanovafundacio.cat</t>
+          <t>info@reusploms.cat</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Club Patí Vilanova</t>
+          <t>CN Reus Ploms (hoquei patins)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Vilanova i la Geltrú</t>
+          <t>Reus</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>santsmontjuic@esportbarrio.com</t>
+          <t>info@cpmanlleu.cat</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Club Sants-Montjuïc Hoquei Patins</t>
+          <t>CP Manlleu (Martinelia)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Manlleu</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>admin@vilassarhoquei.cat</t>
+          <t>coordinador@cpmanlleu.cat</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Club Vilassar Hoquei</t>
+          <t>CP Manlleu (Martinelia)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Vilassar de Mar</t>
+          <t>Manlleu</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>esportiu@vilassarhoquei.cat</t>
+          <t>info@cpvoltrega.com</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Club Vilassar Hoquei</t>
+          <t>CP Voltregà</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Vilassar de Mar</t>
+          <t>Les Masies de Voltregà</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>web@vilassarhoquei.cat</t>
+          <t>cpsantceloni@cpsantceloni.cat</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Club Vilassar Hoquei</t>
+          <t>CPA Sant Celoni</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Vilassar de Mar</t>
+          <t>Sant Celoni</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>sponsors@vilassarhoquei.cat</t>
+          <t>escola@cpisagrera.cat</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Club Vilassar Hoquei</t>
+          <t>CPI La Sagrera</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Vilassar de Mar</t>
+          <t>Barcelona</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>equipacions@vilassarhoquei.cat</t>
+          <t>escola.patinatge@fcbarcelona.cat</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Club Vilassar Hoquei</t>
+          <t>FC Barcelona (hoquei patins)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Vilassar de Mar</t>
+          <t>Barcelona</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>info@reusploms.cat</t>
+          <t>hoqueigeieg@fecapa.cat</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CN Reus Ploms (hoquei patins)</t>
+          <t>GEiEG (hoquei patins)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Reus</t>
+          <t>Girona</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>actividades@reusploms.cat</t>
+          <t>info.gironaclubhoquei@gmail.com</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>CN Reus Ploms (hoquei patins)</t>
+          <t>Girona Club Hoquei</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Reus</t>
+          <t>Girona</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>info@cpmanlleu.cat</t>
+          <t>gironaclubhoquei@fecapa.cat</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>CP Manlleu (Martinelia)</t>
+          <t>Girona Club Hoquei</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Manlleu</t>
+          <t>Girona</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>coordinador@cpmanlleu.cat</t>
+          <t>info.sfericok@gmail.com</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CP Manlleu (Martinelia)</t>
+          <t>HC Sferic Terrassa</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Manlleu</t>
+          <t>Terrassa</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>info@cpvoltrega.com</t>
+          <t>amunthoquei@amunthoquei.cat</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CP Voltregà</t>
+          <t>Hoquei Arenys de Munt</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Les Masies de Voltregà</t>
+          <t>Arenys de Munt</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>cpsantceloni@cpsantceloni.cat</t>
+          <t>hoquei.alpicat@gmail.com</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CPA Sant Celoni</t>
+          <t>Hoquei Club Alpicat</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Sant Celoni</t>
+          <t>Alpicat</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>escola@cpisagrera.cat</t>
+          <t>info@hoqueiclubmontbui.cat</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>CPI La Sagrera</t>
+          <t>Hoquei Club Montbui</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Santa Margarida de Montbui</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>escola.patinatge@fcbarcelona.cat</t>
+          <t>hcpalau@hcpalau.cat</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>FC Barcelona (hoquei patins)</t>
+          <t>Hoquei Club Palau</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Palau-solità i Plegamans</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>hoqueigeieg@fecapa.cat</t>
+          <t>hoqueiclubpiera@gmail.com</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>GEiEG (hoquei patins)</t>
+          <t>Hoquei Club Piera</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Piera</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>info.gironaclubhoquei@gmail.com</t>
+          <t>hcripoll@gmail.com</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Girona Club Hoquei</t>
+          <t>Hoquei Club Ripoll</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Ripoll</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>gironaclubhoquei@fecapa.cat</t>
+          <t>hoqueisalt@gmail.com</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Girona Club Hoquei</t>
+          <t>Hoquei Club Salt</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Salt</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>info.sfericok@gmail.com</t>
+          <t>club@hcsantjust.net</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>HC Sferic Terrassa</t>
+          <t>Hoquei Club Sant Just</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Terrassa</t>
+          <t>Sant Just Desvern</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>amunthoquei@amunthoquei.cat</t>
+          <t>hcsentmenat.junta@gmail.com</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Hoquei Arenys de Munt</t>
+          <t>Hoquei Club Sentmenat</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Arenys de Munt</t>
+          <t>Sentmenat</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>hoquei.alpicat@gmail.com</t>
+          <t>hoqueiclubvalls@gmail.com</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Hoquei Club Alpicat</t>
+          <t>Hoquei Club Valls</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Alpicat</t>
+          <t>Valls</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>info@hoqueiclubmontbui.cat</t>
+          <t>secretaria.ampa@santandreu.manyanet.org</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Hoquei Club Montbui</t>
+          <t>Hoquei JMJ (Col·legi Manyanet Sant Andreu)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Santa Margarida de Montbui</t>
+          <t>Barcelona</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>hcpalau@hcpalau.cat</t>
+          <t>hoquei.patins.tona@gmail.com</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Hoquei Club Palau</t>
+          <t>Hoquei Patins Tona</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Palau-solità i Plegamans</t>
+          <t>Tona</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>hoqueiclubpiera@gmail.com</t>
+          <t>secretaria@igualadahc.com</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Hoquei Club Piera</t>
+          <t>Igualada Hoquei Club</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Piera</t>
+          <t>Igualada</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>hcripoll@gmail.com</t>
+          <t>mollethc@mollethc.cat</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Hoquei Club Ripoll</t>
+          <t>Mollet HC</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Ripoll</t>
+          <t>Mollet del Vallès</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>hoqueisalt@gmail.com</t>
+          <t>info@hoqueitarrega.com</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Hoquei Club Salt</t>
+          <t>Tàrrega Hoquei Patins Club</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Salt</t>
+          <t>Tàrrega</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>club@hcsantjust.net</t>
+          <t>uehorta@uehorta.cat</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Hoquei Club Sant Just</t>
+          <t>UE Horta (hoquei patins)</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Sant Just Desvern</t>
+          <t>Barcelona</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>hcsentmenat.junta@gmail.com</t>
+          <t>uelagarriga@gmail.com</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Hoquei Club Sentmenat</t>
+          <t>UE La Garriga (hoquei)</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Sentmenat</t>
+          <t>La Garriga</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>hoqueiclubvalls@gmail.com</t>
+          <t>lluism1968@gmail.com</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Hoquei Club Valls</t>
+          <t>UE La Garriga (hoquei)</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
-        <is>
-          <t>Valls</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>secretaria.ampa@santandreu.manyanet.org</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Hoquei JMJ (Col·legi Manyanet Sant Andreu)</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>hoquei.patins.tona@gmail.com</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Hoquei Patins Tona</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Tona</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>secretaria@igualadahc.com</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Igualada Hoquei Club</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Igualada</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>mollethc@mollethc.cat</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Mollet HC</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>Mollet del Vallès</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>santcugat-ok.campus@hotmail.com</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Patí Hoquei Club Sant Cugat</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Sant Cugat del Vallès</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>info@hoqueitarrega.com</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Tàrrega Hoquei Patins Club</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Tàrrega</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>uehorta@uehorta.cat</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>UE Horta (hoquei patins)</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>uelagarriga@gmail.com</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>UE La Garriga (hoquei)</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>La Garriga</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>lluism1968@gmail.com</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>UE La Garriga (hoquei)</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
         <is>
           <t>La Garriga</t>
         </is>

</xml_diff>